<commit_message>
feat: implement modular pruning framework with core registry, plugins, pipelines, and evaluation modules
</commit_message>
<xml_diff>
--- a/benchmarks/taylor_benchmark_results.xlsx
+++ b/benchmarks/taylor_benchmark_results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Model Name</t>
   </si>
@@ -61,7 +61,13 @@
     <t>Speedup (%)</t>
   </si>
   <si>
+    <t>Baseline (YOLOv5s)</t>
+  </si>
+  <si>
     <t>Taylor Expansion Pruned</t>
+  </si>
+  <si>
+    <t>weights/yolov5s.pt</t>
   </si>
   <si>
     <t>weights/yolov5s-taylor-pruned.pt</t>
@@ -396,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:15">
@@ -451,46 +457,93 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2">
+        <v>7225885</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>16.436</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0.6627999999999999</v>
+      </c>
+      <c r="H2">
+        <v>0.5503</v>
+      </c>
+      <c r="I2">
+        <v>0.5904</v>
+      </c>
+      <c r="J2">
+        <v>0.3858</v>
+      </c>
+      <c r="K2">
+        <v>94.94</v>
+      </c>
+      <c r="L2">
+        <v>4.76</v>
+      </c>
+      <c r="M2">
+        <v>99.7</v>
+      </c>
+      <c r="N2">
+        <v>10</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3" t="s">
         <v>16</v>
       </c>
-      <c r="C2">
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3">
         <v>4631770</v>
       </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2">
+      <c r="D3">
+        <v>35.9</v>
+      </c>
+      <c r="E3">
         <v>10.633</v>
       </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
-      <c r="K2">
-        <v>73.81</v>
-      </c>
-      <c r="L2">
-        <v>0.48</v>
-      </c>
-      <c r="M2">
-        <v>74.29000000000001</v>
-      </c>
-      <c r="N2">
-        <v>13.5</v>
-      </c>
-      <c r="O2">
-        <v>0</v>
+      <c r="F3">
+        <v>35.31</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>82.04000000000001</v>
+      </c>
+      <c r="L3">
+        <v>0.32</v>
+      </c>
+      <c r="M3">
+        <v>82.36</v>
+      </c>
+      <c r="N3">
+        <v>12.1</v>
+      </c>
+      <c r="O3">
+        <v>17.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>